<commit_message>
vault backup: 2026-03-14 12:22:09
</commit_message>
<xml_diff>
--- a/Курсы/Домашняя работа/Домашняя работа 3/Домашняя работа 3.xlsx
+++ b/Курсы/Домашняя работа/Домашняя работа 3/Домашняя работа 3.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\obsidian-dvfu\Курсы\Домашняя работа\Домашняя работа 3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\obsidian-dvfu\Курсы\Домашняя работа\Домашняя работа 3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43B29ECD-12F3-48A5-BFBD-CC55B81DCD2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91553F83-4836-40D4-8E28-F8FCC95ADDB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10950" yWindow="0" windowWidth="17955" windowHeight="17385" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Описание + особенности аудитори" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>Вводные курса</t>
   </si>
@@ -130,28 +130,6 @@
   </si>
   <si>
     <t>Какие сложности могут возникнуть при работе с данной группой (целевой аудиторией)?</t>
-  </si>
-  <si>
-    <t>Зачем автору (вузу/кафедре): Актуализировать содержание образования под требования цифровой экономики, повысить конкурентоспособность выпускников на рынке труда, укрепить связи с индустриальными партнерами (которым нужны инженеры с навыками Data Science).
-Общая задача курса: Сформировать у студентов системное понимание возможностей и ограничений методов ИИ, а также практические навыки их применения для решения типовых инженерных задач (прогнозирование, классификация, оптимизация).
-Какие образовательные цели закрывает: Курс направлен на формирование универсальных (цифровая культура) и общепрофессиональных компетенций (способность использовать современные IT-технологии в профессиональной деятельности). Он закрывает разрыв между фундаментальной математической подготовкой и реальными запросами работодателей.</t>
-  </si>
-  <si>
-    <t>Студенты останутся на уровне «пользователей» готовых программных продуктов и не смогут самостоятельно разрабатывать или адаптировать алгоритмы ИИ под специфику своей специальности. В результате:
-• В дипломных проектах они не смогут использовать современные методы анализа данных, что снизит качество и актуальность ВКР.
-• При трудоустройстве они проиграют кандидатам, владеющим инструментарием Data Science, даже на традиционных инженерных позициях (где сейчас требуются навыки работы с данными).
-• У них не сформируется системное мышление в области цифровых двойников и предиктивной аналитики, что критично для современной индустрии</t>
-  </si>
-  <si>
-    <t>Знания:
-• Основные типы задач машинного обучения (регрессия, классификация, кластеризация).
-• Архитектуры нейросетей: полносвязные, сверточные (CNN) для работы с сигналами/изображениями, рекуррентные (RNN) для временных рядов.
-• Методы предобработки и нормализации данных, борьба с переобучением.
-Навыки:
-• Программировать на Python с использованием библиотек NumPy, Pandas, Matplotlib, Scikit-learn, PyTorch/TensorFlow.
-• Загружать, анализировать и визуализировать инженерные данные (например, показания датчиков, изображения дефектов).
-• Обучать нейросеть, подбирать гиперпараметры, оценивать качество модели с помощью метрик.
-• Сохранять обученную модель и использовать её для предсказаний на новых данных.</t>
   </si>
   <si>
     <t>• Программирование: Python: типы данных, условные операторы, циклы, функции, работа с файлами, основы ООП.
@@ -170,15 +148,187 @@
 6. Синдром "бумажного инженера": привычка решать задачи аналитически, а не через итеративный эксперимент.</t>
   </si>
   <si>
-    <t>• Минимальный уровень: Студент способен загрузить данные, обучить простую модель по готовому шаблону и интерпретировать результат.
-• Базовый уровень: Студент может самостоятельно выбрать тип модели под задачу, провести предобработку, обучить и оценить качество, исправить типичные ошибки.
-• Продвинутый уровень: Студент способен разработать кастомную архитектуру, оптимизировать гиперпараметры, представить работающий прототип для инженерной задачи и защитить его как мини-проект.
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;Times New Roman&quot;"/>
+        <charset val="204"/>
+      </rPr>
+      <t>Зачем автору (вузу/кафедре):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;Times New Roman&quot;"/>
+      </rPr>
+      <t xml:space="preserve"> Актуализировать содержание образования под требования цифровой экономики, повысить конкурентоспособность выпускников на рынке труда, укрепить связи с индустриальными партнерами (которым нужны инженеры с навыками Data Science).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;Times New Roman&quot;"/>
+        <charset val="204"/>
+      </rPr>
+      <t>Общая задача курса</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;Times New Roman&quot;"/>
+      </rPr>
+      <t xml:space="preserve">: Сформировать у студентов системное понимание возможностей и ограничений методов ИИ, а также практические навыки их применения для решения типовых инженерных задач (прогнозирование, классификация, оптимизация).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;Times New Roman&quot;"/>
+        <charset val="204"/>
+      </rPr>
+      <t>Какие образовательные цели закрывает:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;Times New Roman&quot;"/>
+      </rPr>
+      <t xml:space="preserve"> Курс направлен на формирование универсальных (цифровая культура) и общепрофессиональных компетенций (способность использовать современные IT-технологии в профессиональной деятельности). Он закрывает разрыв между фундаментальной математической подготовкой и реальными запросами работодателей.</t>
+    </r>
+  </si>
+  <si>
+    <t>Студенты останутся на уровне «пользователей» готовых программных продуктов и не смогут самостоятельно разрабатывать или адаптировать алгоритмы ИИ под специфику своей специальности. В результате:
+• В дипломных проектах они не смогут использовать современные методы анализа данных, что снизит качество и актуальность ВКР.
+• При трудоустройстве они проиграют кандидатам, владеющим инструментарием Data Science, даже на традиционных инженерных позициях (где сейчас требуются навыки работы с данными).
+• У них не сформируется системное мышление в области цифровых двойников и предиктивной аналитики, что критично для современной индустрии.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;Times New Roman&quot;"/>
+        <charset val="204"/>
+      </rPr>
+      <t>Знания:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;Times New Roman&quot;"/>
+      </rPr>
+      <t xml:space="preserve">
+• Основные типы задач машинного обучения (регрессия, классификация, кластеризация).
+• Архитектуры нейросетей: полносвязные, сверточные (CNN) для работы с сигналами/изображениями, рекуррентные (RNN) для временных рядов.
+• Методы предобработки и нормализации данных, борьба с переобучением.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;Times New Roman&quot;"/>
+        <charset val="204"/>
+      </rPr>
+      <t>Навыки:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;Times New Roman&quot;"/>
+      </rPr>
+      <t xml:space="preserve">
+• Программировать на Python с использованием библиотек NumPy, Pandas, Matplotlib, Scikit-learn, PyTorch/TensorFlow.
+• Загружать, анализировать и визуализировать инженерные данные (например, показания датчиков, изображения дефектов).
+• Обучать нейросеть, подбирать гиперпараметры, оценивать качество модели с помощью метрик.
+• Сохранять обученную модель и использовать её для предсказаний на новых данных.</t>
+    </r>
+  </si>
+  <si>
+    <t>• Основы работы с большими данными: понятие о распределенных вычислениях (например, Spark), так как многие инженерные данные большие.
+• Основы MLOps: как развернуть модель в production (простое API на Flask/FastAPI), контейнеризация (Docker) — для дальнейшего изучения DevOps и промышленной разработки.
+• Углубленные архитектуры нейросетей: трансформеры, генеративно-состязательные сети (GAN) — для тех, кто пойдет в научные исследования или R&amp;D.
+• Интерпретируемость моделей: методы объяснения предсказаний (SHAP, LIME) — для курсов по надежности и безопасности технических систем.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;Times New Roman&quot;"/>
+        <charset val="204"/>
+      </rPr>
+      <t>Минимальный уровень:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;Times New Roman&quot;"/>
+      </rPr>
+      <t xml:space="preserve"> Студент способен загрузить данные, обучить простую модель по готовому шаблону и интерпретировать результат.
+• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;Times New Roman&quot;"/>
+        <charset val="204"/>
+      </rPr>
+      <t>Базовый уровень:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;Times New Roman&quot;"/>
+      </rPr>
+      <t xml:space="preserve"> Студент может самостоятельно выбрать тип модели под задачу, провести предобработку, обучить и оценить качество, исправить типичные ошибки.
+• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;Times New Roman&quot;"/>
+        <charset val="204"/>
+      </rPr>
+      <t>Продвинутый уровень:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;Times New Roman&quot;"/>
+      </rPr>
+      <t xml:space="preserve"> Студент способен разработать кастомную архитектуру, оптимизировать гиперпараметры, представить работающий прототип для инженерной задачи и защитить его как мини-проект.
 Ожидается, что большинство достигнет базового уровня и сможет использовать нейросети в курсовых и дипломных работах.</t>
-  </si>
-  <si>
-    <t>• Гетерогенность группы: сильные программисты и слабые математики, и наоборот. Преподавателю приходится балансировать между объяснением основ и углубленными темами.
+    </r>
+  </si>
+  <si>
+    <t>• Разнородность группы: сильные программисты и слабые математики, и наоборот. Преподавателю приходится балансировать между объяснением основ и углубленными темами.
 • Высокая загрузка: студенты-инженеры много времени тратят на лабораторные по профильным предметам, поэтому курс не должен требовать более 4-6 часов в неделю самостоятельной работы, иначе они начнут игнорировать задания.
-• Прагматизм: если студент не видит immediate benefit для своей специальности, мотивация падает. Нужно постоянно приводить примеры из их области (механика, электроэнергетика, строительство и т.д.).
+• Прагматизм: если студент не видит применимость темы для своей специальности, мотивация падает. Нужно постоянно приводить примеры из их области (механика, электроэнергетика, строительство и т.д.).
 • Технические проблемы: настройка окружения (установка библиотек, совместимость версий, работа в терминале) может съесть много времени на первых занятиях.
 • Психологический барьер: многие считают нейросети "черным ящиком" и боятся, что не смогут их освоить. Важно развеять этот миф и показывать, что даже простые модели дают полезные результаты.</t>
   </si>
@@ -187,7 +337,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -227,6 +377,19 @@
       <color rgb="FF000000"/>
       <name val="&quot;Times New Roman&quot;"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="&quot;Times New Roman&quot;"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="&quot;Times New Roman&quot;"/>
+      <charset val="204"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -342,26 +505,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -372,6 +520,24 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -655,93 +821,93 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="39.28515625" customWidth="1"/>
-    <col min="2" max="2" width="85.28515625" customWidth="1"/>
+    <col min="1" max="1" width="39.33203125" customWidth="1"/>
+    <col min="2" max="2" width="85.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="24.75" customHeight="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-    </row>
-    <row r="2" spans="1:2" ht="40.5">
-      <c r="A2" s="3" t="s">
+      <c r="B1" s="10"/>
+    </row>
+    <row r="2" spans="1:2" ht="40.799999999999997">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="121.5">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:2" ht="122.4">
+      <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="20.25">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:2" ht="40.799999999999997">
+      <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="40.5">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:2" ht="40.799999999999997">
+      <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="19.5" customHeight="1">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="5"/>
-    </row>
-    <row r="7" spans="1:2" ht="20.25">
-      <c r="A7" s="3" t="s">
+      <c r="B6" s="12"/>
+    </row>
+    <row r="7" spans="1:2" ht="20.399999999999999">
+      <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="1">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="81">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:2" ht="81.599999999999994">
+      <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="303.75">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:2" ht="285.60000000000002">
+      <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="303.75">
-      <c r="A10" s="3" t="s">
+    <row r="10" spans="1:2" ht="306">
+      <c r="A10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="405">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:2" ht="408">
+      <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -757,96 +923,96 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D95ABB7-729F-47F6-AE50-71CE284C9C58}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="29.140625" customWidth="1"/>
-    <col min="2" max="2" width="38.7109375" customWidth="1"/>
-    <col min="3" max="3" width="78.7109375" customWidth="1"/>
+    <col min="1" max="1" width="29.109375" customWidth="1"/>
+    <col min="2" max="2" width="38.6640625" customWidth="1"/>
+    <col min="3" max="3" width="78.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:3" ht="17.399999999999999">
+      <c r="A1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="225">
+    <row r="2" spans="1:3" ht="226.8">
       <c r="A2" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="180">
+      <c r="C2" s="13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="165">
       <c r="A3" s="7"/>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="11" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="255">
+      <c r="C3" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="241.2">
       <c r="A4" s="7"/>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="11" t="s">
-        <v>33</v>
+      <c r="C4" s="13" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="135">
       <c r="A5" s="7"/>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="11" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="135">
+      <c r="C5" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="180">
       <c r="A6" s="7"/>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="11" t="s">
-        <v>34</v>
+      <c r="C6" s="4" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="240">
       <c r="A7" s="7"/>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="165">
+      <c r="C7" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="151.80000000000001">
       <c r="A8" s="7"/>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="11" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="255">
+      <c r="C8" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="240">
       <c r="A9" s="8"/>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="11" t="s">
-        <v>37</v>
+      <c r="C9" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-03-19 10:45:14
</commit_message>
<xml_diff>
--- a/Курсы/Домашняя работа/Домашняя работа 3/Домашняя работа 3.xlsx
+++ b/Курсы/Домашняя работа/Домашняя работа 3/Домашняя работа 3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\obsidian-dvfu\Курсы\Домашняя работа\Домашняя работа 3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91553F83-4836-40D4-8E28-F8FCC95ADDB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C36F458A-692C-44EF-95F6-9665559B3AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Описание + особенности аудитори" sheetId="1" r:id="rId1"/>
@@ -522,11 +522,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -537,9 +535,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -828,10 +828,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="24.75" customHeight="1">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
+      <c r="B1" s="8"/>
     </row>
     <row r="2" spans="1:2" ht="40.799999999999997">
       <c r="A2" s="1" t="s">
@@ -866,10 +866,10 @@
       </c>
     </row>
     <row r="6" spans="1:2" ht="19.5" customHeight="1">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="12"/>
+      <c r="B6" s="10"/>
     </row>
     <row r="7" spans="1:2" ht="20.399999999999999">
       <c r="A7" s="1" t="s">
@@ -903,7 +903,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="408">
+    <row r="11" spans="1:2" ht="409.6">
       <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
@@ -942,18 +942,18 @@
       </c>
     </row>
     <row r="2" spans="1:3" ht="226.8">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="11" t="s">
         <v>22</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="6" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="165">
-      <c r="A3" s="7"/>
+      <c r="A3" s="12"/>
       <c r="B3" s="5" t="s">
         <v>24</v>
       </c>
@@ -962,16 +962,16 @@
       </c>
     </row>
     <row r="4" spans="1:3" ht="241.2">
-      <c r="A4" s="7"/>
+      <c r="A4" s="12"/>
       <c r="B4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="6" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="135">
-      <c r="A5" s="7"/>
+      <c r="A5" s="12"/>
       <c r="B5" s="5" t="s">
         <v>26</v>
       </c>
@@ -980,7 +980,7 @@
       </c>
     </row>
     <row r="6" spans="1:3" ht="180">
-      <c r="A6" s="7"/>
+      <c r="A6" s="12"/>
       <c r="B6" s="5" t="s">
         <v>27</v>
       </c>
@@ -989,7 +989,7 @@
       </c>
     </row>
     <row r="7" spans="1:3" ht="240">
-      <c r="A7" s="7"/>
+      <c r="A7" s="12"/>
       <c r="B7" s="5" t="s">
         <v>28</v>
       </c>
@@ -998,7 +998,7 @@
       </c>
     </row>
     <row r="8" spans="1:3" ht="151.80000000000001">
-      <c r="A8" s="7"/>
+      <c r="A8" s="12"/>
       <c r="B8" s="5" t="s">
         <v>29</v>
       </c>
@@ -1007,7 +1007,7 @@
       </c>
     </row>
     <row r="9" spans="1:3" ht="240">
-      <c r="A9" s="8"/>
+      <c r="A9" s="13"/>
       <c r="B9" s="4" t="s">
         <v>30</v>
       </c>

</xml_diff>